<commit_message>
Djoli reconquete FICTIF v2
</commit_message>
<xml_diff>
--- a/djoli/reconquete/reconquete-clients-inactifs-FICTIF.xlsx
+++ b/djoli/reconquete/reconquete-clients-inactifs-FICTIF.xlsx
@@ -4432,7 +4432,7 @@
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Kra, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Hôtel Ivoire Palm (cuisine), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Kra, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré à l'Hôtel Ivoire Palm (cuisine), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L6" s="16" t="inlineStr"/>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Diallo, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Le Grill du Plateau, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Diallo, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Grill du Plateau, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L8" s="16" t="inlineStr"/>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="K10" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Koffi, c'est Serge de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré au Le Patio d'Angré, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Koffi, c'est Serge de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré au Patio d'Angré, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L10" s="16" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="K14" s="16" t="inlineStr">
         <is>
-          <t>Bonjour Mme Dosso, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Le Comptoir Gourmand, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour Mme Dosso, c'est Aïcha de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Comptoir Gourmand, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L14" s="16" t="inlineStr"/>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="K15" s="20" t="inlineStr">
         <is>
-          <t>Bonjour Mme Brou, c'est Aïcha de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré au Le Jardin de Cocody, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour Mme Brou, c'est Aïcha de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré au Jardin de Cocody, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L15" s="20" t="inlineStr"/>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="K16" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Sylla, c'est Serge de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré au Cantine Entreprise Zone Industrielle, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Sylla, c'est Serge de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré à la Cantine Entreprise Zone Industrielle, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L16" s="16" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Bonjour M. Assi, c'est Aïcha de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré au Le Bistrot du Golf, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Assi, c'est Aïcha de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré au Bistrot du Golf, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L17" s="20" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="K18" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Ahoussou, c'est Aïcha de Djoli. Ça fait 8 semaines qu'on ne vous a pas livré au Hôtel Résidence Akwaba (restaurant), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Ahoussou, c'est Aïcha de Djoli. Ça fait 8 semaines qu'on ne vous a pas livré à l'Hôtel Résidence Akwaba (restaurant), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L18" s="16" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="K19" s="20" t="inlineStr">
         <is>
-          <t>Bonjour Mme Touré, c'est Serge de Djoli. Ça fait 8 semaines qu'on ne vous a pas livré au Cantine Groupe Scolaire Les Palmiers, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour Mme Touré, c'est Serge de Djoli. Ça fait 8 semaines qu'on ne vous a pas livré à la Cantine Groupe Scolaire Les Palmiers, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L19" s="20" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="K20" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Traoré, c'est Serge de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré au Burger &amp; Co Angré, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Traoré, c'est Serge de Djoli. Ça fait 4 semaines qu'on ne vous a pas livré chez Burger &amp; Co Angré, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L20" s="16" t="inlineStr"/>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="K22" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. N'Guessan, c'est Aïcha de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré au La Table de Treichville, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. N'Guessan, c'est Aïcha de Djoli. Ça fait 5 semaines qu'on ne vous a pas livré à la Table de Treichville, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L22" s="16" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="K23" s="20" t="inlineStr">
         <is>
-          <t>Bonjour Mme Kouakou, c'est Mariam de Djoli. Ça fait 7 semaines qu'on ne vous a pas livré au Traiteur Les Délices d'Anoumabo, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour Mme Kouakou, c'est Mariam de Djoli. Ça fait 7 semaines qu'on ne vous a pas livré chez Traiteur Les Délices d'Anoumabo, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L23" s="20" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="K24" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Tanoh, c'est Aïcha de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si le Restaurant Le Vieux Port a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
+          <t>Bonjour M. Tanoh, c'est Aïcha de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si votre établissement a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
         </is>
       </c>
       <c r="L24" s="16" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="K25" s="20" t="inlineStr">
         <is>
-          <t>Bonjour Mme Diabaté, c'est Serge de Djoli. J'espère que tout va bien au Traiteur Mariages &amp; Baptêmes Awa. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
+          <t>Bonjour Mme Diabaté, c'est Serge de Djoli. J'espère que tout va bien chez Traiteur Mariages &amp; Baptêmes Awa. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
         </is>
       </c>
       <c r="L25" s="20" t="inlineStr"/>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="K28" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Gbané, c'est Mariam de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si le Maquis La Paillote a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
+          <t>Bonjour M. Gbané, c'est Mariam de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si votre établissement a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
         </is>
       </c>
       <c r="L28" s="16" t="inlineStr"/>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="K31" s="20" t="inlineStr">
         <is>
-          <t>Bonjour Mme Ehui, c'est Serge de Djoli. J'espère que tout va bien au Pâtisserie-Salon Le Fromager. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
+          <t>Bonjour Mme Ehui, c'est Serge de Djoli. J'espère que tout va bien à la Pâtisserie-Salon Le Fromager. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
         </is>
       </c>
       <c r="L31" s="20" t="inlineStr"/>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="K32" s="16" t="inlineStr">
         <is>
-          <t>Bonjour M. Konan, c'est Mariam de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré au Allocodrome Riviera (stand 12), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour M. Konan, c'est Mariam de Djoli. Ça fait 6 semaines qu'on ne vous a pas livré à l'Allocodrome Riviera (stand 12), je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
       <c r="L32" s="16" t="inlineStr"/>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Bonjour {civ}, c'est {com} de Djoli. Ça fait {sem} semaines qu'on ne vous a pas livré au {etab}, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
+          <t>Bonjour {civ}, c'est {com} de Djoli. Ça fait {sem} semaines qu'on ne vous a pas livré {a_etab}, je voulais simplement prendre de vos nouvelles. Est-ce que quelque chose ne vous a pas convenu de notre côté ? Même deux mots m'aident vraiment.</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6455,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Bonjour {civ}, c'est {com} de Djoli. J'espère que tout va bien au {etab}. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
+          <t>Bonjour {civ}, c'est {com} de Djoli. J'espère que tout va bien {a_etab}. Vous avez un événement ou un gros service en vue ces prochaines semaines ? Je peux vous préparer la liste habituelle à l'avance pour que vous n'ayez qu'à valider.</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>Bonjour {civ}, c'est {com} de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si le {etab} a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
+          <t>Bonjour {civ}, c'est {com} de Djoli. Ça fait un moment qu'on ne s'est pas parlé. Si votre établissement a changé d'organisation ou de fournisseur, aucun souci : j'aimerais juste comprendre ce qui vous a fait partir, pour nous améliorer. Vous auriez deux minutes pour me répondre ?</t>
         </is>
       </c>
     </row>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="D23" s="20" t="inlineStr">
         <is>
-          <t>{civ}, je ne veux pas vous encombrer : je referme le sujet de mon côté. Si le moment change, un simple mot suffit et je reviens vers vous. Bonne continuation au {etab}.</t>
+          <t>{civ}, je ne veux pas vous encombrer : je referme le sujet de mon côté. Si le moment change, un simple mot suffit et je reviens vers vous. Bonne continuation {a_etab}.</t>
         </is>
       </c>
     </row>

</xml_diff>